<commit_message>
feat(inventory): provenance facet with derived counts, detail badge, export and finance columns; the importer stamps importedAt on create
Measured: 1110 unit tests (64 files), 42/42 e2e (import-export.spec.ts + it-core.spec.ts).
</commit_message>
<xml_diff>
--- a/e2e/fixtures/assets-clean.xlsx
+++ b/e2e/fixtures/assets-clean.xlsx
@@ -22,6 +22,9 @@
     <t>Model</t>
   </si>
   <si>
+    <t>Brand</t>
+  </si>
+  <si>
     <t>Serial</t>
   </si>
   <si>
@@ -49,9 +52,18 @@
     <t>Warranty until</t>
   </si>
   <si>
+    <t>Loan until</t>
+  </si>
+  <si>
     <t>Vendor</t>
   </si>
   <si>
+    <t>Provenance</t>
+  </si>
+  <si>
+    <t>Invoice / receipt no.</t>
+  </si>
+  <si>
     <t>RMA ref</t>
   </si>
   <si>
@@ -71,6 +83,9 @@
   </si>
   <si>
     <t>TechServe PH</t>
+  </si>
+  <si>
+    <t>Registered directly</t>
   </si>
   <si>
     <t>imported by the e2e fixture</t>
@@ -152,18 +167,22 @@
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="40" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -209,73 +228,97 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" s="2">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="2">
         <v>46063</v>
       </c>
-      <c r="J2" s="3">
+      <c r="K2" s="3">
         <v>62000</v>
       </c>
-      <c r="K2" s="2">
+      <c r="L2" s="2">
         <v>47159</v>
       </c>
-      <c r="L2" t="s">
-        <v>18</v>
-      </c>
+      <c r="M2" s="2"/>
       <c r="N2" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="O2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="2">
+        <v>46063</v>
+      </c>
+      <c r="K3" s="3">
+        <v>9800</v>
+      </c>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="O3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="2">
-        <v>46063</v>
-      </c>
-      <c r="J3" s="3">
-        <v>9800</v>
-      </c>
-      <c r="K3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="O4" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>